<commit_message>
fix(vision): match dashboard visual layout and dark scale theme with verify_daytime_normal standard
- Use dark background (26, 26, 26) with golden yellow meter ticks (0, 215, 255)
- Standardize header banner with clean English typography (remove broken unicode characters)
- Keep full CCTV resolution without downscaling
- Omit 0.0m tick on staff gauge and display exact water level orange line
</commit_message>
<xml_diff>
--- a/non_time_series/water_levels.xlsx
+++ b/non_time_series/water_levels.xlsx
@@ -514,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -749,6 +749,42 @@
         <v>0.6</v>
       </c>
     </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-01 20:18:15</t>
+        </is>
+      </c>
+      <c r="B19" s="13" t="n">
+        <v>10.19</v>
+      </c>
+      <c r="C19" s="12" t="n"/>
+      <c r="D19" s="12" t="n"/>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-01 20:18:18</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="n"/>
+      <c r="C20" s="10" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="D20" s="9" t="n"/>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-01 20:18:20</t>
+        </is>
+      </c>
+      <c r="B21" s="12" t="n"/>
+      <c r="C21" s="12" t="n"/>
+      <c r="D21" s="13" t="n">
+        <v>0.6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix(vision): align staff gauge calibration, daytime/nighttime baseline detection, and verified benchmark outputs for all 3 stations
</commit_message>
<xml_diff>
--- a/non_time_series/water_levels.xlsx
+++ b/non_time_series/water_levels.xlsx
@@ -514,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -752,7 +752,7 @@
     <row r="19" ht="22" customHeight="1">
       <c r="A19" s="11" t="inlineStr">
         <is>
-          <t>2026-10-01 20:18:15</t>
+          <t>2026-10-01 20:15:53</t>
         </is>
       </c>
       <c r="B19" s="13" t="n">
@@ -764,7 +764,7 @@
     <row r="20" ht="22" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t>2026-10-01 20:18:18</t>
+          <t>2026-10-01 20:15:56</t>
         </is>
       </c>
       <c r="B20" s="9" t="n"/>
@@ -776,7 +776,7 @@
     <row r="21" ht="22" customHeight="1">
       <c r="A21" s="11" t="inlineStr">
         <is>
-          <t>2026-10-01 20:18:20</t>
+          <t>2026-10-01 20:15:58</t>
         </is>
       </c>
       <c r="B21" s="12" t="n"/>
@@ -785,6 +785,78 @@
         <v>0.6</v>
       </c>
     </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-01 22:03:02</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="n">
+        <v>10.08</v>
+      </c>
+      <c r="C22" s="9" t="n"/>
+      <c r="D22" s="9" t="n"/>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-01 22:03:05</t>
+        </is>
+      </c>
+      <c r="B23" s="12" t="n"/>
+      <c r="C23" s="13" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="D23" s="12" t="n"/>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-01 22:03:07</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="n"/>
+      <c r="C24" s="9" t="n"/>
+      <c r="D24" s="10" t="n">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-01 22:04:29</t>
+        </is>
+      </c>
+      <c r="B25" s="13" t="n">
+        <v>10.08</v>
+      </c>
+      <c r="C25" s="12" t="n"/>
+      <c r="D25" s="12" t="n"/>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-01 22:04:32</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="n"/>
+      <c r="C26" s="10" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="D26" s="9" t="n"/>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-01 22:04:34</t>
+        </is>
+      </c>
+      <c r="B27" s="12" t="n"/>
+      <c r="C27" s="12" t="n"/>
+      <c r="D27" s="13" t="n">
+        <v>0.6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
clean(vision): remove unused debug artifacts, temporary outputs, and duplicate sample images
</commit_message>
<xml_diff>
--- a/non_time_series/water_levels.xlsx
+++ b/non_time_series/water_levels.xlsx
@@ -514,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D27"/>
+  <dimension ref="A1:D32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -857,6 +857,66 @@
         <v>0.6</v>
       </c>
     </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-01 22:27:56</t>
+        </is>
+      </c>
+      <c r="B28" s="9" t="n"/>
+      <c r="C28" s="10" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="D28" s="9" t="n"/>
+    </row>
+    <row r="29" ht="22" customHeight="1">
+      <c r="A29" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-01 22:27:59</t>
+        </is>
+      </c>
+      <c r="B29" s="12" t="n"/>
+      <c r="C29" s="12" t="n"/>
+      <c r="D29" s="13" t="n">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-01 22:28:23</t>
+        </is>
+      </c>
+      <c r="B30" s="10" t="n">
+        <v>9.960000000000001</v>
+      </c>
+      <c r="C30" s="9" t="n"/>
+      <c r="D30" s="9" t="n"/>
+    </row>
+    <row r="31" ht="22" customHeight="1">
+      <c r="A31" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-01 22:28:26</t>
+        </is>
+      </c>
+      <c r="B31" s="12" t="n"/>
+      <c r="C31" s="13" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="D31" s="12" t="n"/>
+    </row>
+    <row r="32" ht="22" customHeight="1">
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-01 22:28:27</t>
+        </is>
+      </c>
+      <c r="B32" s="9" t="n"/>
+      <c r="C32" s="9" t="n"/>
+      <c r="D32" s="10" t="n">
+        <v>0.6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>